<commit_message>
Atualização automática: emergencias (07/08/2026 11:16)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/historico_completo_emergencias.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/historico_completo_emergencias.xlsx
@@ -45885,7 +45885,7 @@
         <v>2728</v>
       </c>
       <c r="H580" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="I580" t="s">
         <v>1246</v>
@@ -45909,10 +45909,10 @@
         <v>1477</v>
       </c>
       <c r="Q580">
-        <v>-2</v>
+        <v>-10</v>
       </c>
       <c r="R580">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="S580" t="s">
         <v>1479</v>
@@ -46290,7 +46290,7 @@
         <v>2733</v>
       </c>
       <c r="H586" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="I586" t="s">
         <v>1244</v>

</xml_diff>